<commit_message>
auto: 2026-07-13 13:52 (52件)
</commit_message>
<xml_diff>
--- a/01_プロジェクト/BUYMA購入者配布資料/BUYMA_VIP交渉管理表_購入者版.xlsx
+++ b/01_プロジェクト/BUYMA購入者配布資料/BUYMA_VIP交渉管理表_購入者版.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VIP交渉管理" sheetId="1" r:id="R03d922fae7bb4fc4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使い方" sheetId="2" r:id="Rc8c5ae79e79d48fc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="交渉履歴" sheetId="3" r:id="R6fcb1f3ac6ab4c44"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VIP交渉管理" sheetId="1" r:id="R347b82cf8b194179"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使い方" sheetId="2" r:id="R236eee0dafda4260"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="交渉履歴" sheetId="3" r:id="R25442f7c45de4cd9"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>